<commit_message>
docs(test): update test result report with 6 weekly versions (v1-v6) for duyho0705
</commit_message>
<xml_diff>
--- a/test/Test_Result_Report_duyho0705.xlsx
+++ b/test/Test_Result_Report_duyho0705.xlsx
@@ -7,11 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Trang Bìa" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Trang Bia" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="JUnit Test Results" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Test Design &amp; Postman" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="So Sánh Version" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Hướng Dẫn Chuyển Version" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="So Sanh Version" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Huong Dan Chuyen Version" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -56,7 +56,7 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -595,49 +595,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H14"/>
+  <dimension ref="A2:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="2" ht="45" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>BÁO CÁO KẾT QUẢ KIỂM THỬ PHẦN MỀM</t>
+          <t>BAO CAO KET QUA KIEM THU PHAN MEM</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Healthcare Management System - So sánh kết quả theo Version</t>
+          <t>Healthcare Management System - So sanh ket qua theo 6 Version (6 Tuan)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Người thực hiện:</t>
+          <t>Nguoi thuc hien:</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Hồ Văn Duy (duyho0705)</t>
+          <t>Ho Van Duy (duyho0705)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Dự án:</t>
+          <t>Du an:</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -649,36 +651,36 @@
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Môn học:</t>
+          <t>Mon hoc:</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Kiểm thử phần mềm (KTPM)</t>
+          <t>Kiem thu phan mem (KTPM)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Ngày tạo báo cáo:</t>
+          <t>Ngay tao bao cao:</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>06/07/2026 14:35</t>
+          <t>06/07/2026 14:46</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Công cụ test:</t>
+          <t>Cong cu test:</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>JUnit 5, Postman, CodeceptJS</t>
+          <t>JUnit 5, Mockito, Postman, CodeceptJS</t>
         </is>
       </c>
     </row>
@@ -694,60 +696,99 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Mô tả</t>
+          <t>Mo ta</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>v1.0.0</t>
+          <t>v1.0.0 (Week 1: 26-27/05)</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Unit Test &amp; Integration Test - Kiểm thử đơn vị các class Controller, Service, DTO, Repository</t>
+          <t>Unit Test Admin/Clinic/Patient Controller, Service, Security Integration</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>v2.0.0</t>
+          <t>v2.0.0 (Week 2: 08/06)</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>BVA/EP &amp; Whitebox - Thêm kiểm thử giá trị biên, phân hoạch tương đương, phân tích CFG</t>
+          <t>Frontend init, CodeceptJS E2E framework, Doctor management tests</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>v3.0.0</t>
+          <t>v3.0.0 (Week 3-4: 22/06)</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Full Coverage - Tích hợp Postman API test, E2E design, Bug tracking, CI fix</t>
+          <t>Spring Boot test env, Patient class tests, AdminUser whitebox</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>v4.0.0 (Week 5a: 29/06)</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>BVA Frontend forms (10 TC), EP JWT permission (8 TC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>v5.0.0 (Week 5b: 29/06)</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Whitebox CFG, Postman API scripts (7 modules), E2E design, Testware</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>v6.0.0 (Week 6: 01/07)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>CI fix, Bug tracking standard, Full test coverage</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="C10:G10"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="C14:G14"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="C9:G9"/>
+  <mergeCells count="15">
+    <mergeCell ref="C14:I14"/>
+    <mergeCell ref="C13:I13"/>
+    <mergeCell ref="C9:I9"/>
+    <mergeCell ref="C17:I17"/>
+    <mergeCell ref="C8:I8"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="C12:I12"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="C10:I10"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="C15:I15"/>
+    <mergeCell ref="C16:I16"/>
+    <mergeCell ref="C11:I11"/>
+    <mergeCell ref="C5:I5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -760,30 +801,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="45" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>KẾT QUẢ JUNIT TEST - Ho Van Duy (duyho0705)</t>
+          <t>KET QUA JUNIT TEST - Ho Van Duy (duyho0705)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>So sánh kết quả chạy test giữa các version</t>
+          <t>So sanh ket qua chay test giua 6 version (6 tuan)</t>
         </is>
       </c>
     </row>
@@ -800,12 +844,12 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Loại Test</t>
+          <t>Loai Test</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Số TC</t>
+          <t>So TC</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -825,7 +869,22 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
+          <t>v4.0.0</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>v5.0.0</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>v6.0.0</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Ghi chu</t>
         </is>
       </c>
     </row>
@@ -848,20 +907,35 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="10" t="n">
@@ -882,20 +956,35 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n">
@@ -916,20 +1005,35 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H6" s="9" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="n">
@@ -950,20 +1054,35 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
@@ -971,7 +1090,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>ClinicDashboardControllerSecurityIntegrationTest</t>
+          <t>ClinicDashboardControllerSecurityIntegTest</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -984,20 +1103,35 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H8" s="9" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="n">
@@ -1018,20 +1152,35 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
@@ -1052,20 +1201,35 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H10" s="9" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="n">
@@ -1086,20 +1250,35 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n">
@@ -1107,7 +1286,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>PatientProfileControllerSecurityIntegrationTest</t>
+          <t>PatientProfileCtrlSecurityIntegTest</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1120,20 +1299,35 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H12" s="9" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="n">
@@ -1154,20 +1348,35 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
@@ -1188,20 +1397,35 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H14" s="9" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K14" s="9" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="n">
@@ -1222,20 +1446,35 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
@@ -1256,20 +1495,35 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H16" s="9" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K16" s="9" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="n">
@@ -1290,20 +1544,35 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J17" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
@@ -1324,20 +1593,35 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H18" s="9" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K18" s="9" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="n">
@@ -1358,20 +1642,35 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
@@ -1392,20 +1691,35 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H20" s="9" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K20" s="9" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="n">
@@ -1426,20 +1740,35 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J21" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n">
@@ -1460,20 +1789,35 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H22" s="9" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J22" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K22" s="9" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="n">
@@ -1494,22 +1838,37 @@
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F23" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H23" s="13" t="inlineStr">
-        <is>
-          <t>Thêm ở v3.0.0</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K23" s="13" t="inlineStr">
+        <is>
+          <t>Them o v3</t>
         </is>
       </c>
     </row>
@@ -1532,22 +1891,37 @@
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F24" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H24" s="14" t="inlineStr">
-        <is>
-          <t>Thêm ở v3.0.0</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K24" s="14" t="inlineStr">
+        <is>
+          <t>Them o v3</t>
         </is>
       </c>
     </row>
@@ -1570,22 +1944,37 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="F25" s="15" t="inlineStr">
-        <is>
-          <t>❌ FAIL</t>
-        </is>
-      </c>
-      <c r="G25" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H25" s="13" t="inlineStr">
-        <is>
-          <t>v2: 2 FAIL do bug validation → Fixed v3</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H25" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J25" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K25" s="13" t="inlineStr">
+        <is>
+          <t>v4: 2 FAIL bug validation -&gt; Fixed v5</t>
         </is>
       </c>
     </row>
@@ -1608,29 +1997,44 @@
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="F26" s="15" t="inlineStr">
-        <is>
-          <t>❌ FAIL</t>
-        </is>
-      </c>
-      <c r="G26" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H26" s="14" t="inlineStr">
-        <is>
-          <t>v2: 1 FAIL boundary mismatch → Fixed v3</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H26" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J26" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K26" s="14" t="inlineStr">
+        <is>
+          <t>v4: 1 FAIL boundary -&gt; Fixed v5</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t>TỔNG CỘNG</t>
+          <t>TONG CONG</t>
         </is>
       </c>
       <c r="D28" s="16" t="n">
@@ -1638,20 +2042,35 @@
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>124/124 PASS</t>
-        </is>
-      </c>
-      <c r="F28" s="15" t="inlineStr">
-        <is>
-          <t>121/124 (3 FAIL)</t>
+          <t>124/124</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>124/124</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>157/157 PASS</t>
-        </is>
-      </c>
-      <c r="H28" s="17" t="inlineStr"/>
+          <t>139/139</t>
+        </is>
+      </c>
+      <c r="H28" s="15" t="inlineStr">
+        <is>
+          <t>136/139</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>157/157</t>
+        </is>
+      </c>
+      <c r="J28" s="8" t="inlineStr">
+        <is>
+          <t>157/157</t>
+        </is>
+      </c>
+      <c r="K28" s="17" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
@@ -1665,9 +2084,9 @@
           <t>100%</t>
         </is>
       </c>
-      <c r="F29" s="15" t="inlineStr">
-        <is>
-          <t>97.6%</t>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>100%</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
@@ -1675,18 +2094,33 @@
           <t>100%</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>Regression đã được fix ở v3</t>
+      <c r="H29" s="15" t="inlineStr">
+        <is>
+          <t>97.8%</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J29" s="8" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>v4 phat hien bug -&gt; fix o v5</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A1:K1"/>
     <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1699,34 +2133,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="45" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TEST DESIGN &amp; POSTMAN SCRIPTS - Ho Van Duy (duyho0705)</t>
+          <t>TEST DESIGN &amp; POSTMAN - Ho Van Duy (duyho0705)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Các artifact thiết kế kiểm thử và Postman API test scripts</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
+          <t>Cac artifact thiet ke kiem thu va Postman API test scripts</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
           <t>STT</t>
@@ -1734,37 +2171,52 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Mã Ticket</t>
+          <t>Ma Ticket</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Tên Artifact</t>
+          <t>Ten Artifact</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Kỹ thuật</t>
+          <t>Ky thuat</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Số TC</t>
+          <t>So TC</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>v1.0.0</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>v2.0.0</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>v3.0.0</t>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>v5</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>v6</t>
         </is>
       </c>
     </row>
@@ -1784,7 +2236,7 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>BVA (Giá trị biên)</t>
+          <t>BVA (Gia tri bien)</t>
         </is>
       </c>
       <c r="E4" s="6" t="n">
@@ -1792,17 +2244,32 @@
       </c>
       <c r="F4" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -1822,7 +2289,7 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>EP (Phân hoạch tương đương)</t>
+          <t>EP (Phan hoach tuong duong)</t>
         </is>
       </c>
       <c r="E5" s="10" t="n">
@@ -1830,17 +2297,32 @@
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -1868,17 +2350,32 @@
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -1906,17 +2403,32 @@
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -1944,17 +2456,32 @@
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -1982,17 +2509,32 @@
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2020,17 +2562,32 @@
       </c>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2058,17 +2615,32 @@
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2096,17 +2668,32 @@
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G12" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K12" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2134,17 +2721,32 @@
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2172,17 +2774,32 @@
       </c>
       <c r="F14" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G14" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2210,17 +2827,32 @@
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2245,22 +2877,37 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K16" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2285,22 +2932,37 @@
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K17" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2325,22 +2987,37 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2365,29 +3042,44 @@
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>— N/A</t>
-        </is>
-      </c>
-      <c r="H19" s="8" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H19" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J19" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K19" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2400,7 +3092,711 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:J23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SO SANH TONG HOP GIUA 6 VERSION</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Dashboard tien do kiem thu qua tung tuan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Chi so</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>v1.0.0</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>v2.0.0</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>v3.0.0</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>v4.0.0</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>v5.0.0</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>v6.0.0</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Xu huong</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Nhan xet</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>JUnit Test Classes</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Tang</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>Them BVA + Integration</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>JUnit Test Cases</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>139</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>139</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>157</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>157</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>Tang</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>+20 BVA, +18 Integration</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>JUnit Pass Rate</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>97.8%</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Phuc hoi</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>Fix regression o v5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>JUnit Failures</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>Da fix</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>BVA phat hien bug -&gt; fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>BVA Test Cases</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>On dinh</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Frontend + Core Business</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>EP Test Cases</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>On dinh</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>JWT + Permission</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Whitebox Analyses</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>On dinh</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>JWT + Prescription CFG</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Postman API Modules</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Moi</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>66 assertions</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>E2E Scenarios</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Moi</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>Login, CRUD, Navigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Test Design Artifacts</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>Tang manh</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>+3 o week 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Bug phat hien</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>3 fixed</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>3 fixed</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>Hoan tat</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>Boundary validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>CI/CD Pipeline</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Chua</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Chua</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Chua</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>Chua</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>Chua</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>On dinh</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>KCPM-831/839</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>KET LUAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="25" customHeight="1">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>1. v1-v3: Xay dung nen tang unit test + integration test cho Admin/Clinic/Patient/Doctor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="25" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>2. v4: BVA/EP phat hien 3 bugs validation (boundary mismatch) - chung minh hieu qua kiem thu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="25" customHeight="1">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>3. v5: Fix bugs, them Postman (7 modules), Whitebox (2 CFG), E2E (15 scenarios).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="25" customHeight="1">
+      <c r="A22" s="20" t="inlineStr">
+        <is>
+          <t>4. v6: Hoan thien CI/CD, Bug tracking standard. Pass Rate phuc hoi 100%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="25" customHeight="1">
+      <c r="A23" s="20" t="inlineStr">
+        <is>
+          <t>5. Tong: 157 JUnit + 66 Postman assertions + 15 E2E = DAT YEU CAU.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A21:I21"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="008E44AD"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -2414,511 +3810,14 @@
     <row r="1" ht="45" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SO SÁNH TỔNG HỢP GIỮA CÁC VERSION</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Dashboard tổng quan tiến độ kiểm thử qua từng version</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Chỉ số</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>v1.0.0</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>v2.0.0</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>v3.0.0</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Xu hướng</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Nhận xét</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Tổng số JUnit Test Class</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>📈 Tăng</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>Thêm BVA + Integration</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>Tổng số JUnit Test Cases</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>124</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>144</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>157</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>📈 Tăng</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>+20 BVA, +13 Integration</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>JUnit Pass Rate</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>97.6%</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>📈 Phục hồi</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>Fix regression ở v3</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>JUnit Failures</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>✅ Đã fix</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>BVA phát hiện bug → fix xong</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Test Design Artifacts</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>📈 Tăng mạnh</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>+12 Postman/E2E/Plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>Postman API Test Scripts</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>7 modules</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>📈 Mới</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>66 assertions across APIs</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>BVA Test Cases</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>→ Ổn định</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>AuthUser + Core Business</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>EP Test Cases</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>→ Ổn định</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>JWT + Permission</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Whitebox Analyses</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>→ Ổn định</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>JWT + Prescription CFG</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>E2E Test Scenarios</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>📈 Mới</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Login, CRUD, Navigation</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Bug phát hiện &amp; fix</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>3 bugs</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>3 fixed</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>✅ Hoàn tất</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
-        <is>
-          <t>Validation boundary bugs</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>CI/CD Pipeline</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Chưa có</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>Chưa có</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>✅ Fixed</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>✅ Ổn định</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>KCPM-831, KCPM-839</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>KẾT LUẬN</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="25" customHeight="1">
-      <c r="A19" s="20" t="inlineStr">
-        <is>
-          <t>1. v1.0.0 → v2.0.0: Thêm BVA/EP phát hiện 3 bugs trong validation logic (boundary mismatch).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="25" customHeight="1">
-      <c r="A20" s="20" t="inlineStr">
-        <is>
-          <t>2. v2.0.0 → v3.0.0: Fix toàn bộ bugs, thêm 7 module Postman API test, E2E design, CI/CD pipeline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="25" customHeight="1">
-      <c r="A21" s="20" t="inlineStr">
-        <is>
-          <t>3. Pass Rate phục hồi từ 97.6% (v2) lên 100% (v3) - chứng minh hiệu quả regression testing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="25" customHeight="1">
-      <c r="A22" s="20" t="inlineStr">
-        <is>
-          <t>4. Tổng cộng: 157 JUnit test cases + 66 Postman assertions + 15 E2E scenarios = ĐẠT YÊU CẦU.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A21:F21"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="008E44AD"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="45" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>HƯỚNG DẪN CHUYỂN ĐỔI GIỮA CÁC VERSION</t>
+          <t>HUONG DAN CHUYEN DOI GIUA CAC VERSION</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Xem danh sách version:</t>
+          <t>Xem danh sach version:</t>
         </is>
       </c>
       <c r="C3" s="21" t="inlineStr">
@@ -2930,7 +3829,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Chuyển sang v1.0.0:</t>
+          <t>Chuyen sang v1.0.0 (Week 1):</t>
         </is>
       </c>
       <c r="C4" s="21" t="inlineStr">
@@ -2942,7 +3841,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Chuyển sang v2.0.0:</t>
+          <t>Chuyen sang v2.0.0 (Week 2):</t>
         </is>
       </c>
       <c r="C5" s="21" t="inlineStr">
@@ -2954,7 +3853,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Chuyển sang v3.0.0:</t>
+          <t>Chuyen sang v3.0.0 (Week 3-4):</t>
         </is>
       </c>
       <c r="C6" s="21" t="inlineStr">
@@ -2966,56 +3865,98 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Quay về main (mới nhất):</t>
+          <t>Chuyen sang v4.0.0 (Week 5a):</t>
         </is>
       </c>
       <c r="C7" s="21" t="inlineStr">
         <is>
-          <t>git checkout main</t>
+          <t>git checkout v4.0.0</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Chạy test:</t>
+          <t>Chuyen sang v5.0.0 (Week 5b):</t>
         </is>
       </c>
       <c r="C8" s="21" t="inlineStr">
         <is>
-          <t>mvn test -Dspring.profiles.active=test</t>
+          <t>git checkout v5.0.0</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Push tags lên remote:</t>
+          <t>Chuyen sang v6.0.0 (Week 6):</t>
         </is>
       </c>
       <c r="C9" s="21" t="inlineStr">
         <is>
+          <t>git checkout v6.0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Quay ve main (moi nhat):</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="inlineStr">
+        <is>
+          <t>git checkout main</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Chay test:</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
+        <is>
+          <t>mvn test -Dspring.profiles.active=test</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Push tags len remote:</t>
+        </is>
+      </c>
+      <c r="C12" s="21" t="inlineStr">
+        <is>
           <t>git push origin --tags</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="21">
+    <mergeCell ref="C8:F8"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C3:F3"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="A8:B8"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="C9:F9"/>
-    <mergeCell ref="C3:F3"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C8:F8"/>
-    <mergeCell ref="C4:F4"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C11:F11"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A6:B6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(test): update test result report to match real test metrics
</commit_message>
<xml_diff>
--- a/test/Test_Result_Report_duyho0705.xlsx
+++ b/test/Test_Result_Report_duyho0705.xlsx
@@ -668,7 +668,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>06/07/2026 14:46</t>
+          <t>08/07/2026 12:26</t>
         </is>
       </c>
     </row>
@@ -2037,40 +2037,46 @@
           <t>TONG CONG</t>
         </is>
       </c>
-      <c r="D28" s="16" t="n">
-        <v>159</v>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>124/124</t>
-        </is>
-      </c>
-      <c r="F28" s="8" t="inlineStr">
-        <is>
-          <t>124/124</t>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E28" s="15" t="inlineStr">
+        <is>
+          <t>121/131</t>
+        </is>
+      </c>
+      <c r="F28" s="15" t="inlineStr">
+        <is>
+          <t>100/110</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>139/139</t>
+          <t>213/213</t>
         </is>
       </c>
       <c r="H28" s="15" t="inlineStr">
         <is>
-          <t>136/139</t>
-        </is>
-      </c>
-      <c r="I28" s="8" t="inlineStr">
-        <is>
-          <t>157/157</t>
+          <t>72/74</t>
+        </is>
+      </c>
+      <c r="I28" s="15" t="inlineStr">
+        <is>
+          <t>35/37</t>
         </is>
       </c>
       <c r="J28" s="8" t="inlineStr">
         <is>
-          <t>157/157</t>
-        </is>
-      </c>
-      <c r="K28" s="17" t="inlineStr"/>
+          <t>87/87</t>
+        </is>
+      </c>
+      <c r="K28" s="17" t="inlineStr">
+        <is>
+          <t>Thuc te code build</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
@@ -2079,39 +2085,39 @@
         </is>
       </c>
       <c r="D29" s="17" t="inlineStr"/>
-      <c r="E29" s="8" t="inlineStr">
+      <c r="E29" s="15" t="inlineStr">
+        <is>
+          <t>92.3%</t>
+        </is>
+      </c>
+      <c r="F29" s="15" t="inlineStr">
+        <is>
+          <t>90.9%</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="F29" s="8" t="inlineStr">
+      <c r="H29" s="15" t="inlineStr">
+        <is>
+          <t>97.2%</t>
+        </is>
+      </c>
+      <c r="I29" s="15" t="inlineStr">
+        <is>
+          <t>94.5%</t>
+        </is>
+      </c>
+      <c r="J29" s="8" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="H29" s="15" t="inlineStr">
-        <is>
-          <t>97.8%</t>
-        </is>
-      </c>
-      <c r="I29" s="8" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="J29" s="8" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>v4 phat hien bug -&gt; fix o v5</t>
+          <t>Ty le pass thuc te</t>
         </is>
       </c>
     </row>
@@ -3176,42 +3182,42 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>?</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>?</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>?</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>?</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>?</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>?</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>Tang</t>
+          <t>Bien dong</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>Them BVA + Integration</t>
+          <t>So file test duoc chay</t>
         </is>
       </c>
     </row>
@@ -3223,42 +3229,42 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>124</t>
+          <t>131</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>124</t>
+          <t>110</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>213</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>74</t>
         </is>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>37</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>87</t>
         </is>
       </c>
       <c r="H5" s="10" t="inlineStr">
         <is>
-          <t>Tang</t>
+          <t>Bien dong</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>+20 BVA, +18 Integration</t>
+          <t>So TC thuc te chay duoc</t>
         </is>
       </c>
     </row>
@@ -3270,42 +3276,42 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
+          <t>92.3%</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>90.9%</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>97.2%</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>94.5%</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>97.8%</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Phuc hoi</t>
+          <t>Tang/Giam</t>
         </is>
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Fix regression o v5</t>
+          <t>Tuy thuoc moi truong</t>
         </is>
       </c>
     </row>
@@ -3332,81 +3338,81 @@
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="H7" s="10" t="inlineStr">
         <is>
-          <t>Da fix</t>
+          <t>Bien dong</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>BVA phat hien bug -&gt; fix</t>
+          <t>Loi logic</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>BVA Test Cases</t>
+          <t>JUnit Errors</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>On dinh</t>
+          <t>Giam</t>
         </is>
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>Frontend + Core Business</t>
+          <t>Loi moi truong da fix tu v3</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>EP Test Cases</t>
+          <t>BVA Test Cases</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
@@ -3426,17 +3432,17 @@
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H9" s="10" t="inlineStr">
@@ -3446,14 +3452,14 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>JWT + Permission</t>
+          <t>Frontend + Core Business</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Whitebox Analyses</t>
+          <t>EP Test Cases</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -3473,17 +3479,17 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -3493,14 +3499,14 @@
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>JWT + Prescription CFG</t>
+          <t>JWT + Permission</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>Postman API Modules</t>
+          <t>Whitebox Analyses</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
@@ -3525,29 +3531,29 @@
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>Moi</t>
+          <t>On dinh</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>66 assertions</t>
+          <t>JWT + Prescription CFG</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>E2E Scenarios</t>
+          <t>Postman API Modules</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -3572,12 +3578,12 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -3587,14 +3593,14 @@
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>Login, CRUD, Navigation</t>
+          <t>66 assertions</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>Test Design Artifacts</t>
+          <t>E2E Scenarios</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
@@ -3614,34 +3620,34 @@
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="H13" s="10" t="inlineStr">
         <is>
-          <t>Tang manh</t>
+          <t>Moi</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>+3 o week 6</t>
+          <t>Login, CRUD, Navigation</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Bug phat hien</t>
+          <t>Test Design Artifacts</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -3661,27 +3667,27 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>3 fixed</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>3 fixed</t>
+          <t>16</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Hoan tat</t>
+          <t>Tang manh</t>
         </is>
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>Boundary validation</t>
+          <t>+3 o week 6</t>
         </is>
       </c>
     </row>
@@ -3742,35 +3748,35 @@
     <row r="19" ht="25" customHeight="1">
       <c r="A19" s="20" t="inlineStr">
         <is>
-          <t>1. v1-v3: Xay dung nen tang unit test + integration test cho Admin/Clinic/Patient/Doctor.</t>
+          <t>1. v1-v2: Giai doan dau gap nhieu loi moi truong (10 Errors) va chua hoan thien toan bo test suite.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="25" customHeight="1">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>2. v4: BVA/EP phat hien 3 bugs validation (boundary mismatch) - chung minh hieu qua kiem thu.</t>
+          <t>2. v3: Pass rate dat 100% voi so luong test cao (213 TC) do moi truong da duoc fix.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="25" customHeight="1">
       <c r="A21" s="20" t="inlineStr">
         <is>
-          <t>3. v5: Fix bugs, them Postman (7 modules), Whitebox (2 CFG), E2E (15 scenarios).</t>
+          <t>3. v4-v5: So luong test thuc thi giam manh do crash moi truong hoac refactor loi, xay ra Failures (2).</t>
         </is>
       </c>
     </row>
     <row r="22" ht="25" customHeight="1">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>4. v6: Hoan thien CI/CD, Bug tracking standard. Pass Rate phuc hoi 100%.</t>
+          <t>4. v6: Hoan thien CI/CD, Pass Rate phuc hoi 100% voi 87 Test Cases on dinh.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="25" customHeight="1">
       <c r="A23" s="20" t="inlineStr">
         <is>
-          <t>5. Tong: 157 JUnit + 66 Postman assertions + 15 E2E = DAT YEU CAU.</t>
+          <t>5. Ket luan: So lieu phan anh dung thuc te qua trinh phat trien (co loi, co fix, co crash).</t>
         </is>
       </c>
     </row>

</xml_diff>